<commit_message>
Refresh spec, referentiel and onboarding questionnaire seed
Regenerated seed/onboarding_questionnaire.json from the updated workbook via
scripts/build_seed.py; other seed files were already in sync.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/referentiel_entretien_france.xlsx
+++ b/docs/referentiel_entretien_france.xlsx
@@ -21,7 +21,7 @@
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Equipements!$A$5:$R$112</definedName>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">'Obligations legales'!$A$5:$N$26</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'Plaques par marque'!$A$5:$J$22</definedName>
-    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Questionnaire!$A$5:$L$78</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Questionnaire!$A$5:$L$80</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Taches!$A$5:$O$159</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5171" uniqueCount="2322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5193" uniqueCount="2330">
   <si>
     <t xml:space="preserve">Referentiel d'entretien des equipements du logement - France</t>
   </si>
@@ -5247,7 +5247,7 @@
     <t xml:space="preserve">Questionnaire d'accueil : premiere utilisation et nouveau lieu</t>
   </si>
   <si>
-    <t xml:space="preserve">Une ligne = une reponse possible. Pour chaque obligation créée : date approximative du dernier entretien, ramonage, contrôle ou vidange (mois et année). « Je ne sais pas » la classe « à planifier ».</t>
+    <t xml:space="preserve">Une ligne = une reponse possible. Pour chaque obligation créée, la date du dernier passage (entretien, ramonage, contrôle ou vidange) se donne en chiffres (MM/AAAA). Réponses graduées : date précise → calcul normal ; fait récemment, sans date exacte → à confirmer (orange), avec un rappel pour la préciser ; plus ancien que le délai légal → en retard (rouge) ; jamais réalisé ou je ne sais pas → en retard (rouge), prioritaire.</t>
   </si>
   <si>
     <t xml:space="preserve">Bloc</t>
@@ -5481,7 +5481,7 @@
     <t xml:space="preserve">CUIS-03, CUIS-04</t>
   </si>
   <si>
-    <t xml:space="preserve">Date de péremption imprimée sur le tuyau flexible (une photo suffit).</t>
+    <t xml:space="preserve">Date de péremption imprimée sur le tuyau flexible (MM/AAAA).</t>
   </si>
   <si>
     <t xml:space="preserve">Indice : des brûleurs à flamme signalent une cuisson au gaz.</t>
@@ -5532,7 +5532,7 @@
     <t xml:space="preserve">Voiture</t>
   </si>
   <si>
-    <t xml:space="preserve">Date de première immatriculation et du dernier contrôle technique (photo de la carte grise possible).</t>
+    <t xml:space="preserve">Date de première immatriculation (sur la carte grise) et du dernier contrôle technique (MM/AAAA).</t>
   </si>
   <si>
     <t xml:space="preserve">Moto, scooter ou quadricycle</t>
@@ -5553,7 +5553,7 @@
     <t xml:space="preserve">Ajouté d'office</t>
   </si>
   <si>
-    <t xml:space="preserve">Est-il installé ? Photographiez la date imprimée au dos pour le rappel de remplacement à 10 ans.</t>
+    <t xml:space="preserve">Est-il installé ? Si oui, notez la date de fabrication imprimée au dos (MM/AAAA) : elle fixe son remplacement, 10 ans après.</t>
   </si>
   <si>
     <t xml:space="preserve">Obligatoire dans tout logement : il n'y a pas de question à poser.</t>
@@ -5571,7 +5571,7 @@
     <t xml:space="preserve">Pour chaque obligation créée</t>
   </si>
   <si>
-    <t xml:space="preserve">Pour chaque obligation créée : date approximative du dernier entretien, ramonage, contrôle ou vidange (mois et année). « Je ne sais pas » la classe « à planifier ».</t>
+    <t xml:space="preserve">Pour chaque obligation créée, la date du dernier passage (entretien, ramonage, contrôle ou vidange) se donne en chiffres (MM/AAAA). Réponses graduées : date précise → calcul normal ; fait récemment, sans date exacte → à confirmer (orange), avec un rappel pour la préciser ; plus ancien que le délai légal → en retard (rouge) ; jamais réalisé ou je ne sais pas → en retard (rouge), prioritaire.</t>
   </si>
   <si>
     <t xml:space="preserve">REGLE-02</t>
@@ -5584,6 +5584,30 @@
   </si>
   <si>
     <t xml:space="preserve">« Je ne sais pas » ne bloque jamais la progression : la réponse ajoute un point « à vérifier » sur l'écran d'accueil, avec l'aide associée pour trouver la réponse. Même règle pour les questions de suivi. À l'écran, c'est un choix discret, sous les autres.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REGLE-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Appareil et conduit de fumée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pour chaque réponse créant un appareil et son conduit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quand une réponse crée un appareil à combustion et son conduit de fumée (poêle, insert, chaudière), une seule question de date couvre les deux : l'entretien et le ramonage se font au même passage. Un lien « faits séparément ? » permet de donner deux dates, ou d'indiquer que seul l'un des deux a été fait.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REGLE-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type de logement déjà connu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pour la question Q01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La question Q01 n'est pas posée si le type de logement a déjà été renseigné à la création du lieu.</t>
   </si>
   <si>
     <t xml:space="preserve">Q20</t>
@@ -22014,7 +22038,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:L78"/>
+  <dimension ref="A2:L80"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -23940,7 +23964,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="16" t="s">
         <v>1841</v>
       </c>
@@ -24016,103 +24040,103 @@
         <v>153</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="24" t="s">
+    <row r="57" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="16" t="s">
         <v>1850</v>
       </c>
-      <c r="B57" s="24" t="s">
+      <c r="B57" s="16" t="s">
+        <v>1766</v>
+      </c>
+      <c r="C57" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="D57" s="18" t="s">
         <v>1851</v>
       </c>
-      <c r="C57" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="D57" s="26" t="s">
+      <c r="E57" s="16" t="s">
+        <v>1843</v>
+      </c>
+      <c r="F57" s="18" t="s">
         <v>1852</v>
       </c>
-      <c r="E57" s="24" t="s">
+      <c r="G57" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="H57" s="19" t="s">
         <v>1853</v>
       </c>
-      <c r="F57" s="26" t="s">
+      <c r="I57" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="J57" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="K57" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="L57" s="19" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="16" t="s">
         <v>1854</v>
       </c>
-      <c r="G57" s="25" t="s">
-        <v>352</v>
-      </c>
-      <c r="H57" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="I57" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="J57" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="K57" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="L57" s="25" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="24" t="s">
-        <v>1850</v>
-      </c>
-      <c r="B58" s="24" t="s">
-        <v>1851</v>
-      </c>
-      <c r="C58" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="D58" s="26" t="s">
-        <v>1852</v>
-      </c>
-      <c r="E58" s="24" t="s">
-        <v>1853</v>
-      </c>
-      <c r="F58" s="26" t="s">
+      <c r="B58" s="16" t="s">
+        <v>1766</v>
+      </c>
+      <c r="C58" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="D58" s="18" t="s">
         <v>1855</v>
       </c>
-      <c r="G58" s="25" t="s">
-        <v>360</v>
-      </c>
-      <c r="H58" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="I58" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="J58" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="K58" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="L58" s="25" t="s">
+      <c r="E58" s="16" t="s">
+        <v>1843</v>
+      </c>
+      <c r="F58" s="18" t="s">
+        <v>1856</v>
+      </c>
+      <c r="G58" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="H58" s="19" t="s">
+        <v>1857</v>
+      </c>
+      <c r="I58" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="J58" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="K58" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="L58" s="19" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B59" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C59" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D59" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E59" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F59" s="26" t="s">
-        <v>384</v>
+        <v>1862</v>
       </c>
       <c r="G59" s="25" t="s">
-        <v>382</v>
+        <v>352</v>
       </c>
       <c r="H59" s="25" t="s">
         <v>153</v>
@@ -24132,25 +24156,25 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B60" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C60" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D60" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E60" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F60" s="26" t="s">
-        <v>1856</v>
+        <v>1863</v>
       </c>
       <c r="G60" s="25" t="s">
-        <v>391</v>
+        <v>360</v>
       </c>
       <c r="H60" s="25" t="s">
         <v>153</v>
@@ -24170,25 +24194,25 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B61" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C61" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D61" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E61" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F61" s="26" t="s">
-        <v>398</v>
+        <v>384</v>
       </c>
       <c r="G61" s="25" t="s">
-        <v>397</v>
+        <v>382</v>
       </c>
       <c r="H61" s="25" t="s">
         <v>153</v>
@@ -24208,25 +24232,25 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B62" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C62" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D62" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E62" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F62" s="26" t="s">
-        <v>1857</v>
+        <v>1864</v>
       </c>
       <c r="G62" s="25" t="s">
-        <v>409</v>
+        <v>391</v>
       </c>
       <c r="H62" s="25" t="s">
         <v>153</v>
@@ -24246,25 +24270,25 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B63" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C63" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D63" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E63" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F63" s="26" t="s">
-        <v>1858</v>
+        <v>398</v>
       </c>
       <c r="G63" s="25" t="s">
-        <v>416</v>
+        <v>397</v>
       </c>
       <c r="H63" s="25" t="s">
         <v>153</v>
@@ -24284,25 +24308,25 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B64" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C64" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D64" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E64" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F64" s="26" t="s">
-        <v>1859</v>
+        <v>1865</v>
       </c>
       <c r="G64" s="25" t="s">
-        <v>334</v>
+        <v>409</v>
       </c>
       <c r="H64" s="25" t="s">
         <v>153</v>
@@ -24322,25 +24346,25 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B65" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C65" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D65" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E65" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F65" s="26" t="s">
-        <v>1860</v>
+        <v>1866</v>
       </c>
       <c r="G65" s="25" t="s">
-        <v>441</v>
+        <v>416</v>
       </c>
       <c r="H65" s="25" t="s">
         <v>153</v>
@@ -24360,25 +24384,25 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B66" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C66" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D66" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E66" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F66" s="26" t="s">
-        <v>1861</v>
+        <v>1867</v>
       </c>
       <c r="G66" s="25" t="s">
-        <v>446</v>
+        <v>334</v>
       </c>
       <c r="H66" s="25" t="s">
         <v>153</v>
@@ -24398,25 +24422,25 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B67" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C67" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D67" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E67" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F67" s="26" t="s">
-        <v>1862</v>
+        <v>1868</v>
       </c>
       <c r="G67" s="25" t="s">
-        <v>453</v>
+        <v>441</v>
       </c>
       <c r="H67" s="25" t="s">
         <v>153</v>
@@ -24436,25 +24460,25 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B68" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C68" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D68" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E68" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F68" s="26" t="s">
-        <v>461</v>
+        <v>1869</v>
       </c>
       <c r="G68" s="25" t="s">
-        <v>460</v>
+        <v>446</v>
       </c>
       <c r="H68" s="25" t="s">
         <v>153</v>
@@ -24474,31 +24498,31 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B69" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C69" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D69" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E69" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F69" s="26" t="s">
-        <v>1863</v>
+        <v>1870</v>
       </c>
       <c r="G69" s="25" t="s">
-        <v>316</v>
+        <v>453</v>
       </c>
       <c r="H69" s="25" t="s">
         <v>153</v>
       </c>
       <c r="I69" s="25" t="s">
-        <v>1864</v>
+        <v>153</v>
       </c>
       <c r="J69" s="25" t="s">
         <v>153</v>
@@ -24512,25 +24536,25 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B70" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C70" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D70" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E70" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F70" s="26" t="s">
-        <v>289</v>
+        <v>461</v>
       </c>
       <c r="G70" s="25" t="s">
-        <v>288</v>
+        <v>460</v>
       </c>
       <c r="H70" s="25" t="s">
         <v>153</v>
@@ -24550,31 +24574,31 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B71" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C71" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D71" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E71" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F71" s="26" t="s">
-        <v>1865</v>
+        <v>1871</v>
       </c>
       <c r="G71" s="25" t="s">
-        <v>647</v>
+        <v>316</v>
       </c>
       <c r="H71" s="25" t="s">
         <v>153</v>
       </c>
       <c r="I71" s="25" t="s">
-        <v>1866</v>
+        <v>1872</v>
       </c>
       <c r="J71" s="25" t="s">
         <v>153</v>
@@ -24588,25 +24612,25 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B72" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C72" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D72" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E72" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F72" s="26" t="s">
-        <v>714</v>
+        <v>289</v>
       </c>
       <c r="G72" s="25" t="s">
-        <v>713</v>
+        <v>288</v>
       </c>
       <c r="H72" s="25" t="s">
         <v>153</v>
@@ -24626,31 +24650,31 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B73" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C73" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D73" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E73" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F73" s="26" t="s">
-        <v>1867</v>
+        <v>1873</v>
       </c>
       <c r="G73" s="25" t="s">
-        <v>694</v>
+        <v>647</v>
       </c>
       <c r="H73" s="25" t="s">
         <v>153</v>
       </c>
       <c r="I73" s="25" t="s">
-        <v>153</v>
+        <v>1874</v>
       </c>
       <c r="J73" s="25" t="s">
         <v>153</v>
@@ -24664,25 +24688,25 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B74" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C74" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D74" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E74" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F74" s="26" t="s">
-        <v>1868</v>
+        <v>714</v>
       </c>
       <c r="G74" s="25" t="s">
-        <v>789</v>
+        <v>713</v>
       </c>
       <c r="H74" s="25" t="s">
         <v>153</v>
@@ -24702,25 +24726,25 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B75" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C75" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D75" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E75" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F75" s="26" t="s">
-        <v>799</v>
+        <v>1875</v>
       </c>
       <c r="G75" s="25" t="s">
-        <v>798</v>
+        <v>694</v>
       </c>
       <c r="H75" s="25" t="s">
         <v>153</v>
@@ -24740,31 +24764,31 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B76" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C76" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D76" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E76" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F76" s="26" t="s">
-        <v>1869</v>
+        <v>1876</v>
       </c>
       <c r="G76" s="25" t="s">
-        <v>1870</v>
+        <v>789</v>
       </c>
       <c r="H76" s="25" t="s">
         <v>153</v>
       </c>
       <c r="I76" s="25" t="s">
-        <v>1871</v>
+        <v>153</v>
       </c>
       <c r="J76" s="25" t="s">
         <v>153</v>
@@ -24778,25 +24802,25 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B77" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C77" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D77" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E77" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F77" s="26" t="s">
-        <v>1872</v>
+        <v>799</v>
       </c>
       <c r="G77" s="25" t="s">
-        <v>603</v>
+        <v>798</v>
       </c>
       <c r="H77" s="25" t="s">
         <v>153</v>
@@ -24816,44 +24840,120 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="24" t="s">
-        <v>1850</v>
+        <v>1858</v>
       </c>
       <c r="B78" s="24" t="s">
-        <v>1851</v>
+        <v>1859</v>
       </c>
       <c r="C78" s="24" t="n">
         <v>20</v>
       </c>
       <c r="D78" s="26" t="s">
-        <v>1852</v>
+        <v>1860</v>
       </c>
       <c r="E78" s="24" t="s">
-        <v>1853</v>
+        <v>1861</v>
       </c>
       <c r="F78" s="26" t="s">
-        <v>1873</v>
+        <v>1877</v>
       </c>
       <c r="G78" s="25" t="s">
+        <v>1878</v>
+      </c>
+      <c r="H78" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="I78" s="25" t="s">
+        <v>1879</v>
+      </c>
+      <c r="J78" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="K78" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="L78" s="25" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="24" t="s">
+        <v>1858</v>
+      </c>
+      <c r="B79" s="24" t="s">
+        <v>1859</v>
+      </c>
+      <c r="C79" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="D79" s="26" t="s">
+        <v>1860</v>
+      </c>
+      <c r="E79" s="24" t="s">
+        <v>1861</v>
+      </c>
+      <c r="F79" s="26" t="s">
+        <v>1880</v>
+      </c>
+      <c r="G79" s="25" t="s">
+        <v>603</v>
+      </c>
+      <c r="H79" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="I79" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="J79" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="K79" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="L79" s="25" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="24" t="s">
+        <v>1858</v>
+      </c>
+      <c r="B80" s="24" t="s">
+        <v>1859</v>
+      </c>
+      <c r="C80" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="D80" s="26" t="s">
+        <v>1860</v>
+      </c>
+      <c r="E80" s="24" t="s">
+        <v>1861</v>
+      </c>
+      <c r="F80" s="26" t="s">
+        <v>1881</v>
+      </c>
+      <c r="G80" s="25" t="s">
         <v>838</v>
       </c>
-      <c r="H78" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="I78" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="J78" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="K78" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="L78" s="25" t="s">
+      <c r="H80" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="I80" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="J80" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="K80" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="L80" s="25" t="s">
         <v>153</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:L78"/>
+  <autoFilter ref="A5:L80"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -24886,349 +24986,349 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>1874</v>
+        <v>1882</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>1875</v>
+        <v>1883</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>1876</v>
+        <v>1884</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>1877</v>
+        <v>1885</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>1878</v>
+        <v>1886</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>1879</v>
+        <v>1887</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>1880</v>
+        <v>1888</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>1881</v>
+        <v>1889</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>1882</v>
+        <v>1890</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>1883</v>
+        <v>1891</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>1884</v>
+        <v>1892</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>1885</v>
+        <v>1893</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>1886</v>
+        <v>1894</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>1887</v>
+        <v>1895</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>1888</v>
+        <v>1896</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>1889</v>
+        <v>1897</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>1890</v>
+        <v>1898</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>1891</v>
+        <v>1899</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>1892</v>
+        <v>1900</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>1893</v>
+        <v>1901</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>1894</v>
+        <v>1902</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>1895</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>1896</v>
+        <v>1904</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>1896</v>
+        <v>1904</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>1897</v>
+        <v>1905</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>1898</v>
+        <v>1906</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>1899</v>
+        <v>1907</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>1901</v>
+        <v>1909</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>1902</v>
+        <v>1910</v>
       </c>
       <c r="I7" s="15" t="s">
+        <v>1911</v>
+      </c>
+      <c r="J7" s="26" t="s">
         <v>1903</v>
-      </c>
-      <c r="J7" s="26" t="s">
-        <v>1895</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>1904</v>
+        <v>1912</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>1904</v>
+        <v>1912</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>1905</v>
+        <v>1913</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>1906</v>
+        <v>1914</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>1907</v>
+        <v>1915</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>1908</v>
+        <v>1916</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>1909</v>
+        <v>1917</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>1910</v>
+        <v>1918</v>
       </c>
       <c r="J8" s="26" t="s">
-        <v>1895</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>1911</v>
+        <v>1919</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>1911</v>
+        <v>1919</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>1912</v>
+        <v>1920</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>1913</v>
+        <v>1921</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>1914</v>
+        <v>1922</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>1915</v>
+        <v>1923</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>1916</v>
+        <v>1924</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>1917</v>
+        <v>1925</v>
       </c>
       <c r="J9" s="26" t="s">
-        <v>1895</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>1918</v>
+        <v>1926</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>1918</v>
+        <v>1926</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>1912</v>
+        <v>1920</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>1919</v>
+        <v>1927</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>1920</v>
+        <v>1928</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>1921</v>
+        <v>1929</v>
       </c>
       <c r="H10" s="15" t="s">
         <v>153</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>1922</v>
+        <v>1930</v>
       </c>
       <c r="J10" s="26" t="s">
-        <v>1895</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>1923</v>
+        <v>1931</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>1924</v>
+        <v>1932</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>1925</v>
+        <v>1933</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>1926</v>
+        <v>1934</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>1927</v>
+        <v>1935</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>1928</v>
+        <v>1936</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>1929</v>
+        <v>1937</v>
       </c>
       <c r="I11" s="15" t="s">
-        <v>1930</v>
+        <v>1938</v>
       </c>
       <c r="J11" s="18" t="s">
-        <v>1931</v>
+        <v>1939</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>1932</v>
+        <v>1940</v>
       </c>
       <c r="B12" s="15" t="s">
+        <v>1941</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>1933</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>1925</v>
-      </c>
       <c r="D12" s="15" t="s">
-        <v>1934</v>
+        <v>1942</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>1935</v>
+        <v>1943</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>1928</v>
+        <v>1936</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>1936</v>
+        <v>1944</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>1937</v>
+        <v>1945</v>
       </c>
       <c r="J12" s="18" t="s">
-        <v>1938</v>
+        <v>1946</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>1939</v>
+        <v>1947</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>1940</v>
+        <v>1948</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>1925</v>
+        <v>1933</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>1941</v>
+        <v>1949</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>1942</v>
+        <v>1950</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>1943</v>
+        <v>1951</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>1944</v>
+        <v>1952</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>1945</v>
+        <v>1953</v>
       </c>
       <c r="J13" s="18" t="s">
-        <v>1946</v>
+        <v>1954</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>1947</v>
+        <v>1955</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>1948</v>
+        <v>1956</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>1949</v>
+        <v>1957</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>1950</v>
+        <v>1958</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>1951</v>
+        <v>1959</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>1952</v>
+        <v>1960</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>1953</v>
+        <v>1961</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>1954</v>
+        <v>1962</v>
       </c>
       <c r="J14" s="18" t="s">
-        <v>1955</v>
+        <v>1963</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>1956</v>
+        <v>1964</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>1957</v>
+        <v>1965</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>1958</v>
+        <v>1966</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>1959</v>
+        <v>1967</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>1960</v>
+        <v>1968</v>
       </c>
       <c r="F15" s="15" t="s">
         <v>153</v>
@@ -25237,36 +25337,36 @@
         <v>181</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>1961</v>
+        <v>1969</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>1962</v>
+        <v>1970</v>
       </c>
       <c r="J15" s="26" t="s">
-        <v>1963</v>
+        <v>1971</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>1964</v>
+        <v>1972</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>1965</v>
+        <v>1973</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>1925</v>
+        <v>1933</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>1966</v>
+        <v>1974</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>153</v>
@@ -25275,30 +25375,30 @@
         <v>153</v>
       </c>
       <c r="J16" s="30" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>1967</v>
+        <v>1975</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>1968</v>
+        <v>1976</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>1925</v>
+        <v>1933</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>1966</v>
+        <v>1974</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>153</v>
@@ -25307,30 +25407,30 @@
         <v>153</v>
       </c>
       <c r="J17" s="30" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>1969</v>
+        <v>1977</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>1970</v>
+        <v>1978</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>1925</v>
+        <v>1933</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>1966</v>
+        <v>1974</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>153</v>
@@ -25339,30 +25439,30 @@
         <v>153</v>
       </c>
       <c r="J18" s="30" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>1971</v>
+        <v>1979</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>1972</v>
+        <v>1980</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>1973</v>
+        <v>1981</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>1974</v>
+        <v>1982</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>153</v>
@@ -25371,59 +25471,59 @@
         <v>153</v>
       </c>
       <c r="J19" s="30" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>1975</v>
+        <v>1983</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>1976</v>
+        <v>1984</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>1977</v>
+        <v>1985</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>1978</v>
+        <v>1986</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>1979</v>
+        <v>1987</v>
       </c>
       <c r="I20" s="15" t="s">
         <v>153</v>
       </c>
       <c r="J20" s="30" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>1980</v>
+        <v>1988</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>1981</v>
+        <v>1989</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>1982</v>
+        <v>1990</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G21" s="15" t="s">
         <v>304</v>
@@ -25435,7 +25535,7 @@
         <v>153</v>
       </c>
       <c r="J21" s="30" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25443,22 +25543,22 @@
         <v>44</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>1983</v>
+        <v>1991</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>1984</v>
+        <v>1992</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>1985</v>
+        <v>1993</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>153</v>
@@ -25467,7 +25567,7 @@
         <v>153</v>
       </c>
       <c r="J22" s="30" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
     </row>
   </sheetData>
@@ -25507,12 +25607,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>1986</v>
+        <v>1994</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>1987</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25520,78 +25620,78 @@
         <v>79</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>1988</v>
+        <v>1996</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>1989</v>
+        <v>1997</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>1990</v>
+        <v>1998</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>1991</v>
+        <v>1999</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>1992</v>
+        <v>2000</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>1993</v>
+        <v>2001</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>1994</v>
+        <v>2002</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>1884</v>
+        <v>1892</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>1995</v>
+        <v>2003</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>1996</v>
+        <v>2004</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>1997</v>
+        <v>2005</v>
       </c>
       <c r="M5" s="9" t="s">
-        <v>1998</v>
+        <v>2006</v>
       </c>
       <c r="N5" s="9" t="s">
-        <v>1999</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>2000</v>
+        <v>2008</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>2001</v>
+        <v>2009</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>2002</v>
+        <v>2010</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>2003</v>
+        <v>2011</v>
       </c>
       <c r="E6" s="15" t="s">
         <v>915</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>2004</v>
+        <v>2012</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>2005</v>
+        <v>2013</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>2006</v>
+        <v>2014</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>2007</v>
+        <v>2015</v>
       </c>
       <c r="J6" s="28" t="s">
         <v>153</v>
       </c>
       <c r="K6" s="28" t="s">
-        <v>2008</v>
+        <v>2016</v>
       </c>
       <c r="L6" s="28" t="s">
         <v>153</v>
@@ -25600,92 +25700,92 @@
         <v>1592</v>
       </c>
       <c r="N6" s="28" t="s">
-        <v>2009</v>
+        <v>2017</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>2010</v>
+        <v>2018</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>2011</v>
+        <v>2019</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>2012</v>
+        <v>2020</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>2013</v>
+        <v>2021</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>2014</v>
+        <v>2022</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>2016</v>
+        <v>2024</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>2017</v>
+        <v>2025</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>2018</v>
+        <v>2026</v>
       </c>
       <c r="J7" s="28" t="s">
-        <v>2019</v>
+        <v>2027</v>
       </c>
       <c r="K7" s="28" t="s">
-        <v>2020</v>
+        <v>2028</v>
       </c>
       <c r="L7" s="28" t="s">
         <v>153</v>
       </c>
       <c r="M7" s="28" t="s">
-        <v>2021</v>
+        <v>2029</v>
       </c>
       <c r="N7" s="28" t="s">
-        <v>2022</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>2023</v>
+        <v>2031</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>2024</v>
+        <v>2032</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>2025</v>
+        <v>2033</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>2026</v>
+        <v>2034</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>2027</v>
+        <v>2035</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>2028</v>
+        <v>2036</v>
       </c>
       <c r="G8" s="15" t="s">
         <v>112</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>2029</v>
+        <v>2037</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>2018</v>
+        <v>2026</v>
       </c>
       <c r="J8" s="28" t="s">
         <v>153</v>
       </c>
       <c r="K8" s="28" t="s">
-        <v>2030</v>
+        <v>2038</v>
       </c>
       <c r="L8" s="28" t="s">
         <v>153</v>
       </c>
       <c r="M8" s="28" t="s">
-        <v>2031</v>
+        <v>2039</v>
       </c>
       <c r="N8" s="28" t="s">
         <v>153</v>
@@ -25693,31 +25793,31 @@
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>2032</v>
+        <v>2040</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>2033</v>
+        <v>2041</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>2034</v>
+        <v>2042</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>2035</v>
+        <v>2043</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>2036</v>
+        <v>2044</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>2037</v>
+        <v>2045</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>112</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>2038</v>
+        <v>2046</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>2039</v>
+        <v>2047</v>
       </c>
       <c r="J9" s="28" t="s">
         <v>153</v>
@@ -25732,37 +25832,37 @@
         <v>153</v>
       </c>
       <c r="N9" s="28" t="s">
-        <v>2040</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>2041</v>
+        <v>2049</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>2042</v>
+        <v>2050</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>2043</v>
+        <v>2051</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>2044</v>
+        <v>2052</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>2045</v>
+        <v>2053</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>2046</v>
+        <v>2054</v>
       </c>
       <c r="G10" s="15" t="s">
+        <v>2055</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>2056</v>
+      </c>
+      <c r="I10" s="15" t="s">
         <v>2047</v>
       </c>
-      <c r="H10" s="15" t="s">
-        <v>2048</v>
-      </c>
-      <c r="I10" s="15" t="s">
-        <v>2039</v>
-      </c>
       <c r="J10" s="28" t="s">
         <v>153</v>
       </c>
@@ -25776,39 +25876,39 @@
         <v>153</v>
       </c>
       <c r="N10" s="28" t="s">
-        <v>2049</v>
+        <v>2057</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>2050</v>
+        <v>2058</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>2051</v>
+        <v>2059</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>2052</v>
+        <v>2060</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>2053</v>
+        <v>2061</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>2054</v>
+        <v>2062</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>2055</v>
+        <v>2063</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>2056</v>
+        <v>2064</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>2057</v>
+        <v>2065</v>
       </c>
       <c r="I11" s="15" t="s">
-        <v>2058</v>
+        <v>2066</v>
       </c>
       <c r="J11" s="28" t="s">
-        <v>2059</v>
+        <v>2067</v>
       </c>
       <c r="K11" s="28" t="s">
         <v>153</v>
@@ -25820,48 +25920,48 @@
         <v>153</v>
       </c>
       <c r="N11" s="28" t="s">
-        <v>2060</v>
+        <v>2068</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>2061</v>
+        <v>2069</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>2062</v>
+        <v>2070</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>2063</v>
+        <v>2071</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>2064</v>
+        <v>2072</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>2065</v>
+        <v>2073</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>2066</v>
+        <v>2074</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>642</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>2067</v>
+        <v>2075</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>2068</v>
+        <v>2076</v>
       </c>
       <c r="J12" s="28" t="s">
         <v>153</v>
       </c>
       <c r="K12" s="28" t="s">
-        <v>2069</v>
+        <v>2077</v>
       </c>
       <c r="L12" s="28" t="s">
         <v>153</v>
       </c>
       <c r="M12" s="28" t="s">
-        <v>2070</v>
+        <v>2078</v>
       </c>
       <c r="N12" s="28" t="s">
         <v>153</v>
@@ -25869,43 +25969,43 @@
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>2071</v>
+        <v>2079</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>2072</v>
+        <v>2080</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>2073</v>
+        <v>2081</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>2074</v>
+        <v>2082</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>2075</v>
+        <v>2083</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>2076</v>
+        <v>2084</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>2077</v>
+        <v>2085</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>2078</v>
+        <v>2086</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>2079</v>
+        <v>2087</v>
       </c>
       <c r="J13" s="28" t="s">
-        <v>2080</v>
+        <v>2088</v>
       </c>
       <c r="K13" s="28" t="s">
         <v>153</v>
       </c>
       <c r="L13" s="28" t="s">
-        <v>2081</v>
+        <v>2089</v>
       </c>
       <c r="M13" s="28" t="s">
-        <v>2082</v>
+        <v>2090</v>
       </c>
       <c r="N13" s="28" t="s">
         <v>153</v>
@@ -25913,31 +26013,31 @@
     </row>
     <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>2083</v>
+        <v>2091</v>
       </c>
       <c r="B14" s="18" t="s">
+        <v>2092</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>2093</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>2094</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>2095</v>
+      </c>
+      <c r="F14" s="15" t="s">
         <v>2084</v>
       </c>
-      <c r="C14" s="15" t="s">
-        <v>2085</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>2086</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>2087</v>
-      </c>
-      <c r="F14" s="15" t="s">
-        <v>2076</v>
-      </c>
       <c r="G14" s="15" t="s">
-        <v>2088</v>
+        <v>2096</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>2089</v>
+        <v>2097</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>2090</v>
+        <v>2098</v>
       </c>
       <c r="J14" s="28" t="s">
         <v>153</v>
@@ -25952,39 +26052,39 @@
         <v>153</v>
       </c>
       <c r="N14" s="28" t="s">
-        <v>2091</v>
+        <v>2099</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>2092</v>
+        <v>2100</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>2093</v>
+        <v>2101</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>2094</v>
+        <v>2102</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>2095</v>
+        <v>2103</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>2096</v>
+        <v>2104</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>2076</v>
+        <v>2084</v>
       </c>
       <c r="G15" s="15" t="s">
-        <v>2097</v>
+        <v>2105</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>2098</v>
+        <v>2106</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>2099</v>
+        <v>2107</v>
       </c>
       <c r="J15" s="28" t="s">
-        <v>2100</v>
+        <v>2108</v>
       </c>
       <c r="K15" s="28" t="s">
         <v>153</v>
@@ -25996,36 +26096,36 @@
         <v>153</v>
       </c>
       <c r="N15" s="28" t="s">
-        <v>2101</v>
+        <v>2109</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>2102</v>
+        <v>2110</v>
       </c>
       <c r="B16" s="18" t="s">
         <v>1669</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>2103</v>
+        <v>2111</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>2104</v>
+        <v>2112</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>2105</v>
+        <v>2113</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>2106</v>
+        <v>2114</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>2107</v>
+        <v>2115</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>2108</v>
+        <v>2116</v>
       </c>
       <c r="I16" s="15" t="s">
-        <v>2109</v>
+        <v>2117</v>
       </c>
       <c r="J16" s="28" t="s">
         <v>153</v>
@@ -26034,42 +26134,42 @@
         <v>153</v>
       </c>
       <c r="L16" s="28" t="s">
-        <v>2110</v>
+        <v>2118</v>
       </c>
       <c r="M16" s="28" t="s">
         <v>153</v>
       </c>
       <c r="N16" s="28" t="s">
-        <v>2111</v>
+        <v>2119</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>2112</v>
+        <v>2120</v>
       </c>
       <c r="B17" s="18" t="s">
+        <v>2121</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>2122</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>2123</v>
+      </c>
+      <c r="E17" s="15" t="s">
         <v>2113</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="F17" s="15" t="s">
         <v>2114</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="G17" s="15" t="s">
         <v>2115</v>
       </c>
-      <c r="E17" s="15" t="s">
-        <v>2105</v>
-      </c>
-      <c r="F17" s="15" t="s">
-        <v>2106</v>
-      </c>
-      <c r="G17" s="15" t="s">
-        <v>2107</v>
-      </c>
       <c r="H17" s="15" t="s">
-        <v>2116</v>
+        <v>2124</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>2109</v>
+        <v>2117</v>
       </c>
       <c r="J17" s="28" t="s">
         <v>153</v>
@@ -26078,42 +26178,42 @@
         <v>153</v>
       </c>
       <c r="L17" s="28" t="s">
-        <v>2110</v>
+        <v>2118</v>
       </c>
       <c r="M17" s="28" t="s">
         <v>153</v>
       </c>
       <c r="N17" s="28" t="s">
-        <v>2111</v>
+        <v>2119</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>2117</v>
+        <v>2125</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>2118</v>
+        <v>2126</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>2119</v>
+        <v>2127</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>2120</v>
+        <v>2128</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>2121</v>
+        <v>2129</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>2046</v>
+        <v>2054</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>2122</v>
+        <v>2130</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>2123</v>
+        <v>2131</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>2124</v>
+        <v>2132</v>
       </c>
       <c r="J18" s="28" t="s">
         <v>153</v>
@@ -26122,54 +26222,54 @@
         <v>153</v>
       </c>
       <c r="L18" s="28" t="s">
-        <v>2125</v>
+        <v>2133</v>
       </c>
       <c r="M18" s="28" t="s">
-        <v>2126</v>
+        <v>2134</v>
       </c>
       <c r="N18" s="28" t="s">
-        <v>2127</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>2128</v>
+        <v>2136</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>2129</v>
+        <v>2137</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>2130</v>
+        <v>2138</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>2131</v>
+        <v>2139</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>2132</v>
+        <v>2140</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>2028</v>
+        <v>2036</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>2133</v>
+        <v>2141</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>2134</v>
+        <v>2142</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>2135</v>
+        <v>2143</v>
       </c>
       <c r="J19" s="28" t="s">
         <v>153</v>
       </c>
       <c r="K19" s="28" t="s">
-        <v>2136</v>
+        <v>2144</v>
       </c>
       <c r="L19" s="28" t="s">
         <v>153</v>
       </c>
       <c r="M19" s="28" t="s">
-        <v>2137</v>
+        <v>2145</v>
       </c>
       <c r="N19" s="28" t="s">
         <v>153</v>
@@ -26177,31 +26277,31 @@
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>2138</v>
+        <v>2146</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>2139</v>
+        <v>2147</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>2140</v>
+        <v>2148</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>2141</v>
+        <v>2149</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>2142</v>
+        <v>2150</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>2046</v>
+        <v>2054</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>2143</v>
+        <v>2151</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>2144</v>
+        <v>2152</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>2145</v>
+        <v>2153</v>
       </c>
       <c r="J20" s="28" t="s">
         <v>153</v>
@@ -26210,42 +26310,42 @@
         <v>153</v>
       </c>
       <c r="L20" s="28" t="s">
-        <v>2146</v>
+        <v>2154</v>
       </c>
       <c r="M20" s="28" t="s">
-        <v>2147</v>
+        <v>2155</v>
       </c>
       <c r="N20" s="28" t="s">
-        <v>2148</v>
+        <v>2156</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>2149</v>
+        <v>2157</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>2150</v>
+        <v>2158</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>2151</v>
+        <v>2159</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>2152</v>
+        <v>2160</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>2153</v>
+        <v>2161</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>2076</v>
+        <v>2084</v>
       </c>
       <c r="G21" s="15" t="s">
         <v>847</v>
       </c>
       <c r="H21" s="15" t="s">
-        <v>2154</v>
+        <v>2162</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>2155</v>
+        <v>2163</v>
       </c>
       <c r="J21" s="28" t="s">
         <v>153</v>
@@ -26260,36 +26360,36 @@
         <v>153</v>
       </c>
       <c r="N21" s="28" t="s">
-        <v>2156</v>
+        <v>2164</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>2157</v>
+        <v>2165</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>2158</v>
+        <v>2166</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>2159</v>
+        <v>2167</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>2160</v>
+        <v>2168</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>2161</v>
+        <v>2169</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>2076</v>
+        <v>2084</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>2162</v>
+        <v>2170</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>2163</v>
+        <v>2171</v>
       </c>
       <c r="I22" s="15" t="s">
-        <v>2164</v>
+        <v>2172</v>
       </c>
       <c r="J22" s="28" t="s">
         <v>153</v>
@@ -26301,39 +26401,39 @@
         <v>153</v>
       </c>
       <c r="M22" s="28" t="s">
-        <v>2165</v>
+        <v>2173</v>
       </c>
       <c r="N22" s="28" t="s">
-        <v>2166</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>2167</v>
+        <v>2175</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>2168</v>
+        <v>2176</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>2169</v>
+        <v>2177</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>2170</v>
+        <v>2178</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>2171</v>
+        <v>2179</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>2172</v>
+        <v>2180</v>
       </c>
       <c r="G23" s="15" t="s">
         <v>227</v>
       </c>
       <c r="H23" s="15" t="s">
-        <v>2173</v>
+        <v>2181</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>2164</v>
+        <v>2172</v>
       </c>
       <c r="J23" s="28" t="s">
         <v>153</v>
@@ -26342,10 +26442,10 @@
         <v>153</v>
       </c>
       <c r="L23" s="28" t="s">
-        <v>2174</v>
+        <v>2182</v>
       </c>
       <c r="M23" s="28" t="s">
-        <v>2175</v>
+        <v>2183</v>
       </c>
       <c r="N23" s="28" t="s">
         <v>153</v>
@@ -26353,31 +26453,31 @@
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>2176</v>
+        <v>2184</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>2177</v>
+        <v>2185</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>2178</v>
+        <v>2186</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>2179</v>
+        <v>2187</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>2180</v>
+        <v>2188</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>2076</v>
+        <v>2084</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>2181</v>
+        <v>2189</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>2182</v>
+        <v>2190</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>2183</v>
+        <v>2191</v>
       </c>
       <c r="J24" s="28" t="s">
         <v>153</v>
@@ -26389,42 +26489,42 @@
         <v>153</v>
       </c>
       <c r="M24" s="28" t="s">
-        <v>2184</v>
+        <v>2192</v>
       </c>
       <c r="N24" s="28" t="s">
-        <v>2185</v>
+        <v>2193</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>2186</v>
+        <v>2194</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>2187</v>
+        <v>2195</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>2188</v>
+        <v>2196</v>
       </c>
       <c r="D25" s="15" t="s">
         <v>872</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>2189</v>
+        <v>2197</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>2190</v>
+        <v>2198</v>
       </c>
       <c r="G25" s="15" t="s">
         <v>875</v>
       </c>
       <c r="H25" s="15" t="s">
-        <v>2191</v>
+        <v>2199</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>2192</v>
+        <v>2200</v>
       </c>
       <c r="J25" s="28" t="s">
-        <v>2193</v>
+        <v>2201</v>
       </c>
       <c r="K25" s="28" t="s">
         <v>153</v>
@@ -26436,27 +26536,27 @@
         <v>153</v>
       </c>
       <c r="N25" s="28" t="s">
-        <v>2194</v>
+        <v>2202</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>2195</v>
+        <v>2203</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>2196</v>
+        <v>2204</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>2197</v>
+        <v>2205</v>
       </c>
       <c r="D26" s="15" t="s">
+        <v>2206</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>2207</v>
+      </c>
+      <c r="F26" s="15" t="s">
         <v>2198</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>2199</v>
-      </c>
-      <c r="F26" s="15" t="s">
-        <v>2190</v>
       </c>
       <c r="G26" s="15" t="s">
         <v>875</v>
@@ -26465,10 +26565,10 @@
         <v>887</v>
       </c>
       <c r="I26" s="15" t="s">
-        <v>2200</v>
+        <v>2208</v>
       </c>
       <c r="J26" s="28" t="s">
-        <v>2193</v>
+        <v>2201</v>
       </c>
       <c r="K26" s="28" t="s">
         <v>153</v>
@@ -26512,26 +26612,26 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>2201</v>
+        <v>2209</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>2202</v>
+        <v>2210</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>2203</v>
+        <v>2211</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>2204</v>
+        <v>2212</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>2205</v>
+        <v>2213</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>2206</v>
+        <v>2214</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26539,7 +26639,7 @@
         <v>35</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>2207</v>
+        <v>2215</v>
       </c>
       <c r="C6" s="21" t="s">
         <v>41</v>
@@ -26551,7 +26651,7 @@
         <v>35</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>2208</v>
+        <v>2216</v>
       </c>
       <c r="C7" s="21" t="s">
         <v>42</v>
@@ -26563,7 +26663,7 @@
         <v>35</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>2209</v>
+        <v>2217</v>
       </c>
       <c r="C8" s="21" t="s">
         <v>43</v>
@@ -26575,7 +26675,7 @@
         <v>35</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>2210</v>
+        <v>2218</v>
       </c>
       <c r="C9" s="21" t="s">
         <v>44</v>
@@ -26587,13 +26687,13 @@
         <v>35</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>2211</v>
+        <v>2219</v>
       </c>
       <c r="C10" s="21" t="s">
         <v>45</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>2212</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26601,7 +26701,7 @@
         <v>35</v>
       </c>
       <c r="B11" s="30" t="s">
-        <v>2213</v>
+        <v>2221</v>
       </c>
       <c r="C11" s="21" t="s">
         <v>46</v>
@@ -26613,7 +26713,7 @@
         <v>35</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>2214</v>
+        <v>2222</v>
       </c>
       <c r="C12" s="21" t="s">
         <v>47</v>
@@ -26625,7 +26725,7 @@
         <v>35</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>2215</v>
+        <v>2223</v>
       </c>
       <c r="C13" s="21" t="s">
         <v>48</v>
@@ -26637,13 +26737,13 @@
         <v>35</v>
       </c>
       <c r="B14" s="30" t="s">
-        <v>2216</v>
+        <v>2224</v>
       </c>
       <c r="C14" s="21" t="s">
         <v>49</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>2217</v>
+        <v>2225</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26651,191 +26751,191 @@
         <v>35</v>
       </c>
       <c r="B15" s="30" t="s">
-        <v>2218</v>
+        <v>2226</v>
       </c>
       <c r="C15" s="21" t="s">
         <v>50</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>2212</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>2219</v>
+        <v>2227</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>2220</v>
+        <v>2228</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>2221</v>
+        <v>2229</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>2222</v>
+        <v>2230</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>2219</v>
+        <v>2227</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>2223</v>
+        <v>2231</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>2224</v>
+        <v>2232</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>2225</v>
+        <v>2233</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>2219</v>
+        <v>2227</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>2226</v>
+        <v>2234</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>2227</v>
+        <v>2235</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>2228</v>
+        <v>2236</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>2229</v>
+        <v>2237</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>2230</v>
+        <v>2238</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>2231</v>
+        <v>2239</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>2232</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>2229</v>
+        <v>2237</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>2233</v>
+        <v>2241</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>2234</v>
+        <v>2242</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>2235</v>
+        <v>2243</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>2229</v>
+        <v>2237</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>2236</v>
+        <v>2244</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>2237</v>
+        <v>2245</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>2238</v>
+        <v>2246</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>2229</v>
+        <v>2237</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>2239</v>
+        <v>2247</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>2240</v>
+        <v>2248</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>2241</v>
+        <v>2249</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>2242</v>
+        <v>2250</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>2243</v>
+        <v>2251</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>2244</v>
+        <v>2252</v>
       </c>
       <c r="D23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>2242</v>
+        <v>2250</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>2245</v>
+        <v>2253</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>2246</v>
+        <v>2254</v>
       </c>
       <c r="D24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>2242</v>
+        <v>2250</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>2247</v>
+        <v>2255</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>2248</v>
+        <v>2256</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>2249</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>2242</v>
+        <v>2250</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>2250</v>
+        <v>2258</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>2251</v>
+        <v>2259</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>2252</v>
+        <v>2260</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>2242</v>
+        <v>2250</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>2253</v>
+        <v>2261</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>2254</v>
+        <v>2262</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>2255</v>
+        <v>2263</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>2242</v>
+        <v>2250</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>2256</v>
+        <v>2264</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>2257</v>
+        <v>2265</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>2258</v>
+        <v>2266</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26843,13 +26943,13 @@
         <v>53</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>2259</v>
+        <v>2267</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>56</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>2260</v>
+        <v>2268</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26857,13 +26957,13 @@
         <v>53</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>2261</v>
+        <v>2269</v>
       </c>
       <c r="C30" s="15" t="s">
         <v>58</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>2262</v>
+        <v>2270</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26871,317 +26971,317 @@
         <v>53</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>2263</v>
+        <v>2271</v>
       </c>
       <c r="C31" s="15" t="s">
         <v>60</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>2264</v>
+        <v>2272</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>2265</v>
+        <v>2273</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>2266</v>
+        <v>2274</v>
       </c>
       <c r="C32" s="15" t="s">
         <v>112</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>2267</v>
+        <v>2275</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>2265</v>
+        <v>2273</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>2268</v>
+        <v>2276</v>
       </c>
       <c r="C33" s="15" t="s">
         <v>149</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>2269</v>
+        <v>2277</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>2265</v>
+        <v>2273</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>2270</v>
+        <v>2278</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>2271</v>
+        <v>2279</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>2272</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="15" t="s">
-        <v>2265</v>
+        <v>2273</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>2273</v>
+        <v>2281</v>
       </c>
       <c r="C35" s="15" t="s">
         <v>227</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>2274</v>
+        <v>2282</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="15" t="s">
-        <v>2265</v>
+        <v>2273</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>2275</v>
+        <v>2283</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>2276</v>
+        <v>2284</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>2277</v>
+        <v>2285</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="15" t="s">
-        <v>2265</v>
+        <v>2273</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>2278</v>
+        <v>2286</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>581</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>2279</v>
+        <v>2287</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="15" t="s">
-        <v>2265</v>
+        <v>2273</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>2280</v>
+        <v>2288</v>
       </c>
       <c r="C38" s="15" t="s">
         <v>779</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>2281</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="15" t="s">
-        <v>2282</v>
+        <v>2290</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>2283</v>
+        <v>2291</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>2284</v>
+        <v>2292</v>
       </c>
       <c r="D39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>2282</v>
+        <v>2290</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>2285</v>
+        <v>2293</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>2286</v>
+        <v>2294</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>2287</v>
+        <v>2295</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>2282</v>
+        <v>2290</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>2288</v>
+        <v>2296</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>2289</v>
+        <v>2297</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>2290</v>
+        <v>2298</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="15" t="s">
-        <v>2282</v>
+        <v>2290</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>2291</v>
+        <v>2299</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>2292</v>
+        <v>2300</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>2293</v>
+        <v>2301</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="15" t="s">
-        <v>2294</v>
+        <v>2302</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>2295</v>
+        <v>2303</v>
       </c>
       <c r="C43" s="15" t="s">
         <v>72</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>2296</v>
+        <v>2304</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="15" t="s">
-        <v>2294</v>
+        <v>2302</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>2297</v>
+        <v>2305</v>
       </c>
       <c r="C44" s="15" t="s">
         <v>73</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>2298</v>
+        <v>2306</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="15" t="s">
-        <v>2294</v>
+        <v>2302</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>2299</v>
+        <v>2307</v>
       </c>
       <c r="C45" s="15" t="s">
         <v>74</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>2300</v>
+        <v>2308</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="15" t="s">
-        <v>2294</v>
+        <v>2302</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>2301</v>
+        <v>2309</v>
       </c>
       <c r="C46" s="15" t="s">
         <v>75</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>2302</v>
+        <v>2310</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="15" t="s">
-        <v>2294</v>
+        <v>2302</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>2303</v>
+        <v>2311</v>
       </c>
       <c r="C47" s="15" t="s">
         <v>76</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>2304</v>
+        <v>2312</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="15" t="s">
-        <v>2305</v>
+        <v>2313</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>2306</v>
+        <v>2314</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>2307</v>
+        <v>2315</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>2308</v>
+        <v>2316</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="15" t="s">
-        <v>2305</v>
+        <v>2313</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>2309</v>
+        <v>2317</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>1955</v>
+        <v>1963</v>
       </c>
       <c r="D49" s="15" t="s">
-        <v>2310</v>
+        <v>2318</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="15" t="s">
-        <v>2305</v>
+        <v>2313</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>2311</v>
+        <v>2319</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>1900</v>
+        <v>1908</v>
       </c>
       <c r="D50" s="15" t="s">
-        <v>2312</v>
+        <v>2320</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="15" t="s">
-        <v>2313</v>
+        <v>2321</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>2314</v>
+        <v>2322</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>2315</v>
+        <v>2323</v>
       </c>
       <c r="D51" s="15" t="s">
-        <v>2316</v>
+        <v>2324</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="15" t="s">
-        <v>2313</v>
+        <v>2321</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>2317</v>
+        <v>2325</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>2318</v>
+        <v>2326</v>
       </c>
       <c r="D52" s="15"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="15" t="s">
-        <v>2313</v>
+        <v>2321</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>2319</v>
+        <v>2327</v>
       </c>
       <c r="C53" s="15" t="s">
-        <v>2320</v>
+        <v>2328</v>
       </c>
       <c r="D53" s="15" t="s">
-        <v>2321</v>
+        <v>2329</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Concentrated dashboard and monthly maintenance guidance
Home now leads with a global status and an overdue-only "À faire
maintenant", with per-place cards linking to a new place page that
holds the full obligations list, this month's lifespan maintenance and
the appliance list. Maintenance tasks get their own fiche (procedure,
DIY/pro, "C'est fait") backed by a new maintenance_completions table
(RLS from creation, covered by test-isolation.mjs). Questionnaire
"jamais"/"je ne sais pas" answers are consolidated into single,
consistently styled buttons.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/referentiel_entretien_france.xlsx
+++ b/docs/referentiel_entretien_france.xlsx
@@ -5246,7 +5246,7 @@
     <t xml:space="preserve">Questionnaire d'accueil : premiere utilisation et nouveau lieu</t>
   </si>
   <si>
-    <t xml:space="preserve">Une ligne = une reponse possible. Chaque obligation a sa propre question de date (onglet Questions de date, seed/date_questions.json), qui nomme l'appareil et l'intervention. Réponses graduées avec le vrai délai de l'obligation : mois et année → calcul normal ; « Il y a moins de {délai} », sans date précise → à confirmer (orange) ; « Il y a plus de {délai} » → en retard (rouge) ; « Jamais » ou « Je ne sais pas » → en retard, prioritaire. Les dates se choisissent dans deux listes (mois en toutes lettres, année) et s'affichent « septembre 2026 », jamais avec un jour.</t>
+    <t xml:space="preserve">Une ligne = une reponse possible. Chaque obligation a sa propre question de date (onglet Questions de date, seed/date_questions.json), qui nomme l'appareil et l'intervention. Réponses graduées avec le vrai délai de l'obligation : mois et année → calcul normal ; « Il y a moins de {délai} », sans date précise → à confirmer (orange) ; « Il y a plus de {délai} » → en retard (rouge) ; « Jamais ou je ne sais pas », un seul bouton en dernière position → en retard, prioritaire. Les dates se choisissent dans deux listes (mois en toutes lettres, année) et s'affichent « septembre 2026 », jamais avec un jour.</t>
   </si>
   <si>
     <t xml:space="preserve">Bloc</t>
@@ -5588,7 +5588,7 @@
     <t xml:space="preserve">Pour chaque obligation créée</t>
   </si>
   <si>
-    <t xml:space="preserve">Chaque obligation a sa propre question de date (onglet Questions de date, seed/date_questions.json), qui nomme l'appareil et l'intervention. Réponses graduées avec le vrai délai de l'obligation : mois et année → calcul normal ; « Il y a moins de {délai} », sans date précise → à confirmer (orange) ; « Il y a plus de {délai} » → en retard (rouge) ; « Jamais » ou « Je ne sais pas » → en retard, prioritaire. Les dates se choisissent dans deux listes (mois en toutes lettres, année) et s'affichent « septembre 2026 », jamais avec un jour.</t>
+    <t xml:space="preserve">Chaque obligation a sa propre question de date (onglet Questions de date, seed/date_questions.json), qui nomme l'appareil et l'intervention. Réponses graduées avec le vrai délai de l'obligation : mois et année → calcul normal ; « Il y a moins de {délai} », sans date précise → à confirmer (orange) ; « Il y a plus de {délai} » → en retard (rouge) ; « Jamais ou je ne sais pas », un seul bouton en dernière position → en retard, prioritaire. Les dates se choisissent dans deux listes (mois en toutes lettres, année) et s'affichent « septembre 2026 », jamais avec un jour.</t>
   </si>
   <si>
     <t xml:space="preserve">REGLE-02</t>
@@ -5600,7 +5600,7 @@
     <t xml:space="preserve">Pour chaque question d'obligation</t>
   </si>
   <si>
-    <t xml:space="preserve">« Je ne sais pas » ne bloque jamais la progression : la réponse ajoute un point « à vérifier » sur l'écran d'accueil, avec l'aide associée pour trouver la réponse. Même règle pour les questions de suivi. À l'écran, c'est un choix discret, sous les autres.</t>
+    <t xml:space="preserve">« Je ne sais pas » ne bloque jamais la progression : la réponse ajoute un point « à vérifier » sur l'écran d'accueil, avec l'aide associée pour trouver la réponse. Même règle pour les questions de suivi. À l'écran, c'est un bouton comme les autres, en dernière position.</t>
   </si>
   <si>
     <t xml:space="preserve">REGLE-03</t>
@@ -5726,7 +5726,7 @@
     <t xml:space="preserve">Une question de date par obligation, avec le vrai delai legal</t>
   </si>
   <si>
-    <t xml:space="preserve">Mois gradue : mois et annee | Il y a moins de {delai} | Il y a plus de {delai} | Jamais | Je ne sais pas. Affichage des dates : septembre 2026.</t>
+    <t xml:space="preserve">Mois gradue : mois et annee | Il y a moins de {delai} | Il y a plus de {delai} | Jamais ou je ne sais pas (un seul bouton, en dernier). Affichage des dates : septembre 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Cle</t>
@@ -24628,7 +24628,7 @@
         <v>1845</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="16" t="s">
         <v>1846</v>
       </c>
@@ -24669,7 +24669,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="16" t="s">
         <v>1851</v>
       </c>

</xml_diff>

<commit_message>
Move three tasks to Essentiel and add the fiche's empty-level state
Refresh spec/referentiel/seed from the "fiche" workbook revision (T-042,
T-045, T-131 now essential). Fills the one gap left in the already-merged
appliance fiche: an appliance with zero maintenance tasks at the place's
current level now says "Aucun geste indispensable pour cet appareil.
Passez au niveau Recommandé pour voir ses N gestes d'entretien." instead
of rendering nothing.

Not yet tested against a live account: the dev server's authenticated
pages currently fail with "Cookies can only be modified in a Server
Action or Route Handler" from auth.getSession() (src/lib/db.ts),
reproducible on main too. Investigating separately.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/referentiel_entretien_france.xlsx
+++ b/docs/referentiel_entretien_france.xlsx
@@ -17237,7 +17237,7 @@
         <v>56</v>
       </c>
       <c r="P47" s="23" t="s">
-        <v>940</v>
+        <v>933</v>
       </c>
       <c r="Q47" s="24" t="n">
         <v>15</v>
@@ -17399,7 +17399,7 @@
         <v>56</v>
       </c>
       <c r="P50" s="23" t="s">
-        <v>940</v>
+        <v>933</v>
       </c>
       <c r="Q50" s="24" t="n">
         <v>30</v>
@@ -22043,7 +22043,7 @@
         <v>56</v>
       </c>
       <c r="P136" s="23" t="s">
-        <v>940</v>
+        <v>933</v>
       </c>
       <c r="Q136" s="24" t="n">
         <v>15</v>

</xml_diff>

<commit_message>
Refresh spec, référentiel and seed for the rendez-vous chantier
Revision 52: rendez-vous pris, never-future "C'est fait", and the smoke
detector's two possible printed dates (fabrication vs. replacement deadline).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/referentiel_entretien_france.xlsx
+++ b/docs/referentiel_entretien_france.xlsx
@@ -5954,7 +5954,7 @@
     <t xml:space="preserve">Péremption</t>
   </si>
   <si>
-    <t xml:space="preserve">Mois et année, ou « Je ne trouve pas la date » (à confirmer). La date donnée devient l'échéance.</t>
+    <t xml:space="preserve">Mois et année, années futures proposées (la date de péremption est à venir), ou « Je ne trouve pas la date » (à confirmer). La date donnée devient l'échéance.</t>
   </si>
   <si>
     <t xml:space="preserve">Détecteur de fumée</t>
@@ -5966,7 +5966,7 @@
     <t xml:space="preserve">Fabrication</t>
   </si>
   <si>
-    <t xml:space="preserve">Explication affichée : un détecteur se remplace 10 ans après sa fabrication. Mois et année, ou « Je ne la trouve pas » (à confirmer). Échéance = date + 10 ans.</t>
+    <t xml:space="preserve">Deux cas, au choix de l'utilisateur : date de fabrication (échéance = date + 10 ans) ou date limite de remplacement, souvent imprimée « à remplacer avant … » (échéance = cette date). Mois et année ; années futures proposées pour la date limite. « Je ne la trouve pas » → à confirmer.</t>
   </si>
   <si>
     <t xml:space="preserve">Quand la voiture a-t-elle passé son dernier contrôle technique ?</t>
@@ -27480,7 +27480,7 @@
         <v>1968</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16" t="s">
         <v>1246</v>
       </c>
@@ -27503,7 +27503,7 @@
         <v>1972</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="s">
         <v>1366</v>
       </c>

</xml_diff>

<commit_message>
Smoke detector card: one title, kind as subtitle, CE check risk and advice
- The three detector kinds are titled « Détecteur de fumée », with the kind
  as the fiche's subtitle (« Détecteur autonome », « Relié à votre alarme »,
  « Relié à votre alarme télésurveillée »), like brand and model elsewhere.
- Workbook: a « Risque affiche » column on Taches replaces the obligation's
  risks on a task's row, and « Conseil si en retard » on Questions de date
  is shown on a red row. T-158 gets « Un détecteur non conforme peut ne pas
  être reconnu par votre assureur » and the advice to replace the detector
  or contact the monitoring provider. Seed regenerated.
- The CE check's « Mettre à jour » asks its question directly (Oui / Non /
  Je ne sais pas), without the tip already shown on the row.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/referentiel_entretien_france.xlsx
+++ b/docs/referentiel_entretien_france.xlsx
@@ -672,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="B2:C25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="31" min="1" max="1"/>
@@ -680,7 +680,6 @@
     <col width="105" customWidth="1" style="31" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="19.7" customHeight="1" s="32">
       <c r="B2" s="33" t="inlineStr">
         <is>
@@ -695,7 +694,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="42" customHeight="1" s="32">
       <c r="B5" s="35" t="inlineStr">
         <is>
@@ -804,7 +802,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="32">
       <c r="B15" s="35" t="inlineStr">
         <is>
@@ -848,7 +845,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="32">
       <c r="B20" s="35" t="inlineStr">
         <is>
@@ -1531,7 +1527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R114"/>
+  <dimension ref="A2:R114"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="31" min="1" max="1"/>
@@ -1551,7 +1547,6 @@
     <col width="44" customWidth="1" style="31" min="16" max="18"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="19.7" customHeight="1" s="32">
       <c r="A2" s="33" t="inlineStr">
         <is>
@@ -1566,7 +1561,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="32">
       <c r="A5" s="41" t="inlineStr">
         <is>
@@ -11374,7 +11368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q163"/>
+  <dimension ref="A2:R163"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="31" min="1" max="2"/>
@@ -11395,7 +11389,6 @@
     <col width="11" customWidth="1" style="31" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="19.7" customHeight="1" s="32">
       <c r="A2" s="33" t="inlineStr">
         <is>
@@ -11410,7 +11403,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="32">
       <c r="A5" s="41" t="inlineStr">
         <is>
@@ -11495,6 +11487,11 @@
       <c r="Q5" s="41" t="inlineStr">
         <is>
           <t>Temps actif (min)</t>
+        </is>
+      </c>
+      <c r="R5" s="41" t="inlineStr">
+        <is>
+          <t>Risque affiche</t>
         </is>
       </c>
     </row>
@@ -11577,6 +11574,11 @@
       <c r="Q6" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R6" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="35.05" customHeight="1" s="32">
       <c r="A7" s="55" t="inlineStr">
@@ -11657,6 +11659,11 @@
       <c r="Q7" s="56" t="n">
         <v>3</v>
       </c>
+      <c r="R7" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="23.85" customHeight="1" s="32">
       <c r="A8" s="45" t="inlineStr">
@@ -11737,6 +11744,11 @@
       <c r="Q8" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R8" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="35.05" customHeight="1" s="32">
       <c r="A9" s="49" t="inlineStr">
@@ -11817,6 +11829,11 @@
       <c r="Q9" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R9" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="23.85" customHeight="1" s="32">
       <c r="A10" s="55" t="inlineStr">
@@ -11897,6 +11914,11 @@
       <c r="Q10" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R10" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="23.85" customHeight="1" s="32">
       <c r="A11" s="49" t="inlineStr">
@@ -11977,6 +11999,11 @@
       <c r="Q11" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R11" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="23.85" customHeight="1" s="32">
       <c r="A12" s="55" t="inlineStr">
@@ -12057,6 +12084,11 @@
       <c r="Q12" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R12" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="23.85" customHeight="1" s="32">
       <c r="A13" s="55" t="inlineStr">
@@ -12137,6 +12169,11 @@
       <c r="Q13" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R13" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="35.05" customHeight="1" s="32">
       <c r="A14" s="55" t="inlineStr">
@@ -12217,6 +12254,11 @@
       <c r="Q14" s="56" t="n">
         <v>25</v>
       </c>
+      <c r="R14" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="23.85" customHeight="1" s="32">
       <c r="A15" s="49" t="inlineStr">
@@ -12297,6 +12339,11 @@
       <c r="Q15" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R15" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="23.85" customHeight="1" s="32">
       <c r="A16" s="45" t="inlineStr">
@@ -12377,6 +12424,11 @@
       <c r="Q16" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R16" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="23.85" customHeight="1" s="32">
       <c r="A17" s="55" t="inlineStr">
@@ -12457,6 +12509,11 @@
       <c r="Q17" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R17" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="23.85" customHeight="1" s="32">
       <c r="A18" s="49" t="inlineStr">
@@ -12537,6 +12594,11 @@
       <c r="Q18" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R18" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="35.05" customHeight="1" s="32">
       <c r="A19" s="49" t="inlineStr">
@@ -12617,6 +12679,11 @@
       <c r="Q19" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R19" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="35.05" customHeight="1" s="32">
       <c r="A20" s="49" t="inlineStr">
@@ -12697,6 +12764,11 @@
       <c r="Q20" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R20" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="23.85" customHeight="1" s="32">
       <c r="A21" s="49" t="inlineStr">
@@ -12777,6 +12849,11 @@
       <c r="Q21" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R21" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="35.05" customHeight="1" s="32">
       <c r="A22" s="49" t="inlineStr">
@@ -12857,6 +12934,11 @@
       <c r="Q22" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R22" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="35.05" customHeight="1" s="32">
       <c r="A23" s="55" t="inlineStr">
@@ -12937,6 +13019,11 @@
       <c r="Q23" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R23" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="23.85" customHeight="1" s="32">
       <c r="A24" s="55" t="inlineStr">
@@ -13017,6 +13104,11 @@
       <c r="Q24" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R24" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="23.85" customHeight="1" s="32">
       <c r="A25" s="55" t="inlineStr">
@@ -13097,6 +13189,11 @@
       <c r="Q25" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R25" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="23.85" customHeight="1" s="32">
       <c r="A26" s="49" t="inlineStr">
@@ -13177,6 +13274,11 @@
       <c r="Q26" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R26" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="35.05" customHeight="1" s="32">
       <c r="A27" s="55" t="inlineStr">
@@ -13257,6 +13359,11 @@
       <c r="Q27" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R27" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="23.85" customHeight="1" s="32">
       <c r="A28" s="55" t="inlineStr">
@@ -13337,6 +13444,11 @@
       <c r="Q28" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R28" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="23.85" customHeight="1" s="32">
       <c r="A29" s="45" t="inlineStr">
@@ -13417,6 +13529,11 @@
       <c r="Q29" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R29" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="23.85" customHeight="1" s="32">
       <c r="A30" s="55" t="inlineStr">
@@ -13497,6 +13614,11 @@
       <c r="Q30" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R30" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="23.85" customHeight="1" s="32">
       <c r="A31" s="45" t="inlineStr">
@@ -13577,6 +13699,11 @@
       <c r="Q31" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R31" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="35.05" customHeight="1" s="32">
       <c r="A32" s="55" t="inlineStr">
@@ -13657,6 +13784,11 @@
       <c r="Q32" s="56" t="n">
         <v>2</v>
       </c>
+      <c r="R32" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="35.05" customHeight="1" s="32">
       <c r="A33" s="45" t="inlineStr">
@@ -13737,6 +13869,11 @@
       <c r="Q33" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R33" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="23.85" customHeight="1" s="32">
       <c r="A34" s="55" t="inlineStr">
@@ -13817,6 +13954,11 @@
       <c r="Q34" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R34" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="23.85" customHeight="1" s="32">
       <c r="A35" s="49" t="inlineStr">
@@ -13897,6 +14039,11 @@
       <c r="Q35" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R35" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="23.85" customHeight="1" s="32">
       <c r="A36" s="55" t="inlineStr">
@@ -13977,6 +14124,11 @@
       <c r="Q36" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R36" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="23.85" customHeight="1" s="32">
       <c r="A37" s="45" t="inlineStr">
@@ -14057,6 +14209,11 @@
       <c r="Q37" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R37" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="23.85" customHeight="1" s="32">
       <c r="A38" s="55" t="inlineStr">
@@ -14137,6 +14294,11 @@
       <c r="Q38" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R38" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="23.85" customHeight="1" s="32">
       <c r="A39" s="55" t="inlineStr">
@@ -14217,6 +14379,11 @@
       <c r="Q39" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R39" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="35.05" customHeight="1" s="32">
       <c r="A40" s="55" t="inlineStr">
@@ -14297,6 +14464,11 @@
       <c r="Q40" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R40" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="23.85" customHeight="1" s="32">
       <c r="A41" s="45" t="inlineStr">
@@ -14377,6 +14549,11 @@
       <c r="Q41" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R41" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="23.85" customHeight="1" s="32">
       <c r="A42" s="55" t="inlineStr">
@@ -14457,6 +14634,11 @@
       <c r="Q42" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R42" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="23.85" customHeight="1" s="32">
       <c r="A43" s="55" t="inlineStr">
@@ -14537,6 +14719,11 @@
       <c r="Q43" s="56" t="n">
         <v>45</v>
       </c>
+      <c r="R43" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="23.85" customHeight="1" s="32">
       <c r="A44" s="55" t="inlineStr">
@@ -14617,6 +14804,11 @@
       <c r="Q44" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R44" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="23.85" customHeight="1" s="32">
       <c r="A45" s="55" t="inlineStr">
@@ -14697,6 +14889,11 @@
       <c r="Q45" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R45" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="23.85" customHeight="1" s="32">
       <c r="A46" s="55" t="inlineStr">
@@ -14777,6 +14974,11 @@
       <c r="Q46" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R46" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="23.85" customHeight="1" s="32">
       <c r="A47" s="55" t="inlineStr">
@@ -14857,6 +15059,11 @@
       <c r="Q47" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R47" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="23.85" customHeight="1" s="32">
       <c r="A48" s="55" t="inlineStr">
@@ -14937,6 +15144,11 @@
       <c r="Q48" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R48" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="23.85" customHeight="1" s="32">
       <c r="A49" s="55" t="inlineStr">
@@ -15017,6 +15229,11 @@
       <c r="Q49" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R49" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="35.05" customHeight="1" s="32">
       <c r="A50" s="55" t="inlineStr">
@@ -15097,6 +15314,11 @@
       <c r="Q50" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R50" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="23.85" customHeight="1" s="32">
       <c r="A51" s="55" t="inlineStr">
@@ -15177,6 +15399,11 @@
       <c r="Q51" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R51" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="23.85" customHeight="1" s="32">
       <c r="A52" s="55" t="inlineStr">
@@ -15257,6 +15484,11 @@
       <c r="Q52" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R52" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="23.85" customHeight="1" s="32">
       <c r="A53" s="55" t="inlineStr">
@@ -15337,6 +15569,11 @@
       <c r="Q53" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R53" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="23.85" customHeight="1" s="32">
       <c r="A54" s="55" t="inlineStr">
@@ -15417,6 +15654,11 @@
       <c r="Q54" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R54" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="23.85" customHeight="1" s="32">
       <c r="A55" s="55" t="inlineStr">
@@ -15497,6 +15739,11 @@
       <c r="Q55" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R55" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="23.85" customHeight="1" s="32">
       <c r="A56" s="55" t="inlineStr">
@@ -15577,6 +15824,11 @@
       <c r="Q56" s="56" t="n">
         <v>2</v>
       </c>
+      <c r="R56" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="23.85" customHeight="1" s="32">
       <c r="A57" s="55" t="inlineStr">
@@ -15657,6 +15909,11 @@
       <c r="Q57" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R57" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="23.85" customHeight="1" s="32">
       <c r="A58" s="55" t="inlineStr">
@@ -15737,6 +15994,11 @@
       <c r="Q58" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R58" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="23.85" customHeight="1" s="32">
       <c r="A59" s="55" t="inlineStr">
@@ -15817,6 +16079,11 @@
       <c r="Q59" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R59" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="23.85" customHeight="1" s="32">
       <c r="A60" s="55" t="inlineStr">
@@ -15897,6 +16164,11 @@
       <c r="Q60" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R60" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="23.85" customHeight="1" s="32">
       <c r="A61" s="55" t="inlineStr">
@@ -15977,6 +16249,11 @@
       <c r="Q61" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R61" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="23.85" customHeight="1" s="32">
       <c r="A62" s="55" t="inlineStr">
@@ -16057,6 +16334,11 @@
       <c r="Q62" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R62" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="23.85" customHeight="1" s="32">
       <c r="A63" s="55" t="inlineStr">
@@ -16137,6 +16419,11 @@
       <c r="Q63" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R63" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="23.85" customHeight="1" s="32">
       <c r="A64" s="55" t="inlineStr">
@@ -16217,6 +16504,11 @@
       <c r="Q64" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R64" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="35.05" customHeight="1" s="32">
       <c r="A65" s="49" t="inlineStr">
@@ -16297,6 +16589,11 @@
       <c r="Q65" s="48" t="n">
         <v>3</v>
       </c>
+      <c r="R65" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="23.85" customHeight="1" s="32">
       <c r="A66" s="55" t="inlineStr">
@@ -16377,6 +16674,11 @@
       <c r="Q66" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R66" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="23.85" customHeight="1" s="32">
       <c r="A67" s="55" t="inlineStr">
@@ -16457,6 +16759,11 @@
       <c r="Q67" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R67" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="23.85" customHeight="1" s="32">
       <c r="A68" s="55" t="inlineStr">
@@ -16537,6 +16844,11 @@
       <c r="Q68" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R68" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="23.85" customHeight="1" s="32">
       <c r="A69" s="55" t="inlineStr">
@@ -16617,6 +16929,11 @@
       <c r="Q69" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R69" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="23.85" customHeight="1" s="32">
       <c r="A70" s="55" t="inlineStr">
@@ -16697,6 +17014,11 @@
       <c r="Q70" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R70" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="32">
       <c r="A71" s="55" t="inlineStr">
@@ -16777,6 +17099,11 @@
       <c r="Q71" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R71" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="35.05" customHeight="1" s="32">
       <c r="A72" s="55" t="inlineStr">
@@ -16857,6 +17184,11 @@
       <c r="Q72" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R72" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="23.85" customHeight="1" s="32">
       <c r="A73" s="45" t="inlineStr">
@@ -16937,6 +17269,11 @@
       <c r="Q73" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R73" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="23.85" customHeight="1" s="32">
       <c r="A74" s="55" t="inlineStr">
@@ -17017,6 +17354,11 @@
       <c r="Q74" s="56" t="n">
         <v>45</v>
       </c>
+      <c r="R74" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="23.85" customHeight="1" s="32">
       <c r="A75" s="55" t="inlineStr">
@@ -17097,6 +17439,11 @@
       <c r="Q75" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R75" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="35.05" customHeight="1" s="32">
       <c r="A76" s="49" t="inlineStr">
@@ -17177,6 +17524,11 @@
       <c r="Q76" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R76" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="23.85" customHeight="1" s="32">
       <c r="A77" s="49" t="inlineStr">
@@ -17257,6 +17609,11 @@
       <c r="Q77" s="48" t="n">
         <v>60</v>
       </c>
+      <c r="R77" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="23.85" customHeight="1" s="32">
       <c r="A78" s="55" t="inlineStr">
@@ -17337,6 +17694,11 @@
       <c r="Q78" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R78" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="23.85" customHeight="1" s="32">
       <c r="A79" s="55" t="inlineStr">
@@ -17417,6 +17779,11 @@
       <c r="Q79" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R79" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="23.85" customHeight="1" s="32">
       <c r="A80" s="49" t="inlineStr">
@@ -17497,6 +17864,11 @@
       <c r="Q80" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R80" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="35.05" customHeight="1" s="32">
       <c r="A81" s="55" t="inlineStr">
@@ -17577,6 +17949,11 @@
       <c r="Q81" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R81" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="23.85" customHeight="1" s="32">
       <c r="A82" s="45" t="inlineStr">
@@ -17657,6 +18034,11 @@
       <c r="Q82" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R82" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="23.85" customHeight="1" s="32">
       <c r="A83" s="55" t="inlineStr">
@@ -17737,6 +18119,11 @@
       <c r="Q83" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R83" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="23.85" customHeight="1" s="32">
       <c r="A84" s="45" t="inlineStr">
@@ -17817,6 +18204,11 @@
       <c r="Q84" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R84" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="35.05" customHeight="1" s="32">
       <c r="A85" s="55" t="inlineStr">
@@ -17897,6 +18289,11 @@
       <c r="Q85" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R85" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="23.85" customHeight="1" s="32">
       <c r="A86" s="55" t="inlineStr">
@@ -17977,6 +18374,11 @@
       <c r="Q86" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R86" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="23.85" customHeight="1" s="32">
       <c r="A87" s="49" t="inlineStr">
@@ -18057,6 +18459,11 @@
       <c r="Q87" s="48" t="n">
         <v>2</v>
       </c>
+      <c r="R87" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="46.25" customHeight="1" s="32">
       <c r="A88" s="49" t="inlineStr">
@@ -18137,6 +18544,11 @@
       <c r="Q88" s="48" t="n">
         <v>15</v>
       </c>
+      <c r="R88" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="23.85" customHeight="1" s="32">
       <c r="A89" s="55" t="inlineStr">
@@ -18217,6 +18629,11 @@
       <c r="Q89" s="56" t="n">
         <v>2</v>
       </c>
+      <c r="R89" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="23.85" customHeight="1" s="32">
       <c r="A90" s="55" t="inlineStr">
@@ -18297,6 +18714,11 @@
       <c r="Q90" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R90" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="23.85" customHeight="1" s="32">
       <c r="A91" s="49" t="inlineStr">
@@ -18377,6 +18799,11 @@
       <c r="Q91" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R91" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="23.85" customHeight="1" s="32">
       <c r="A92" s="49" t="inlineStr">
@@ -18457,6 +18884,11 @@
       <c r="Q92" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R92" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="23.85" customHeight="1" s="32">
       <c r="A93" s="55" t="inlineStr">
@@ -18537,6 +18969,11 @@
       <c r="Q93" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R93" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="23.85" customHeight="1" s="32">
       <c r="A94" s="55" t="inlineStr">
@@ -18617,6 +19054,11 @@
       <c r="Q94" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R94" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="23.85" customHeight="1" s="32">
       <c r="A95" s="55" t="inlineStr">
@@ -18697,6 +19139,11 @@
       <c r="Q95" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R95" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="23.85" customHeight="1" s="32">
       <c r="A96" s="55" t="inlineStr">
@@ -18777,6 +19224,11 @@
       <c r="Q96" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R96" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="23.85" customHeight="1" s="32">
       <c r="A97" s="55" t="inlineStr">
@@ -18857,6 +19309,11 @@
       <c r="Q97" s="56" t="n">
         <v>45</v>
       </c>
+      <c r="R97" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="23.85" customHeight="1" s="32">
       <c r="A98" s="49" t="inlineStr">
@@ -18937,6 +19394,11 @@
       <c r="Q98" s="48" t="n">
         <v>10</v>
       </c>
+      <c r="R98" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="35.05" customHeight="1" s="32">
       <c r="A99" s="55" t="inlineStr">
@@ -19017,6 +19479,11 @@
       <c r="Q99" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R99" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="23.85" customHeight="1" s="32">
       <c r="A100" s="45" t="inlineStr">
@@ -19097,6 +19564,11 @@
       <c r="Q100" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R100" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="23.85" customHeight="1" s="32">
       <c r="A101" s="55" t="inlineStr">
@@ -19177,6 +19649,11 @@
       <c r="Q101" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R101" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="23.85" customHeight="1" s="32">
       <c r="A102" s="55" t="inlineStr">
@@ -19257,6 +19734,11 @@
       <c r="Q102" s="56" t="n">
         <v>120</v>
       </c>
+      <c r="R102" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="23.85" customHeight="1" s="32">
       <c r="A103" s="55" t="inlineStr">
@@ -19337,6 +19819,11 @@
       <c r="Q103" s="56" t="n">
         <v>90</v>
       </c>
+      <c r="R103" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="23.85" customHeight="1" s="32">
       <c r="A104" s="55" t="inlineStr">
@@ -19417,6 +19904,11 @@
       <c r="Q104" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R104" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="23.85" customHeight="1" s="32">
       <c r="A105" s="49" t="inlineStr">
@@ -19497,6 +19989,11 @@
       <c r="Q105" s="48" t="n">
         <v>5</v>
       </c>
+      <c r="R105" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="23.85" customHeight="1" s="32">
       <c r="A106" s="55" t="inlineStr">
@@ -19577,6 +20074,11 @@
       <c r="Q106" s="56" t="n">
         <v>45</v>
       </c>
+      <c r="R106" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="23.85" customHeight="1" s="32">
       <c r="A107" s="55" t="inlineStr">
@@ -19657,6 +20159,11 @@
       <c r="Q107" s="56" t="n">
         <v>60</v>
       </c>
+      <c r="R107" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="23.85" customHeight="1" s="32">
       <c r="A108" s="55" t="inlineStr">
@@ -19737,6 +20244,11 @@
       <c r="Q108" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R108" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="23.85" customHeight="1" s="32">
       <c r="A109" s="55" t="inlineStr">
@@ -19817,6 +20329,11 @@
       <c r="Q109" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R109" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="23.85" customHeight="1" s="32">
       <c r="A110" s="55" t="inlineStr">
@@ -19897,6 +20414,11 @@
       <c r="Q110" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R110" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="23.85" customHeight="1" s="32">
       <c r="A111" s="55" t="inlineStr">
@@ -19977,6 +20499,11 @@
       <c r="Q111" s="56" t="n">
         <v>60</v>
       </c>
+      <c r="R111" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="23.85" customHeight="1" s="32">
       <c r="A112" s="55" t="inlineStr">
@@ -20057,6 +20584,11 @@
       <c r="Q112" s="56" t="n">
         <v>45</v>
       </c>
+      <c r="R112" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="23.85" customHeight="1" s="32">
       <c r="A113" s="55" t="inlineStr">
@@ -20137,6 +20669,11 @@
       <c r="Q113" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R113" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="23.85" customHeight="1" s="32">
       <c r="A114" s="55" t="inlineStr">
@@ -20217,6 +20754,11 @@
       <c r="Q114" s="56" t="n">
         <v>90</v>
       </c>
+      <c r="R114" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="35.05" customHeight="1" s="32">
       <c r="A115" s="55" t="inlineStr">
@@ -20297,6 +20839,11 @@
       <c r="Q115" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R115" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="23.85" customHeight="1" s="32">
       <c r="A116" s="45" t="inlineStr">
@@ -20377,6 +20924,11 @@
       <c r="Q116" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R116" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="23.85" customHeight="1" s="32">
       <c r="A117" s="55" t="inlineStr">
@@ -20457,6 +21009,11 @@
       <c r="Q117" s="56" t="n">
         <v>180</v>
       </c>
+      <c r="R117" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="35.05" customHeight="1" s="32">
       <c r="A118" s="45" t="inlineStr">
@@ -20537,6 +21094,11 @@
       <c r="Q118" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R118" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="23.85" customHeight="1" s="32">
       <c r="A119" s="55" t="inlineStr">
@@ -20617,6 +21179,11 @@
       <c r="Q119" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R119" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="23.85" customHeight="1" s="32">
       <c r="A120" s="55" t="inlineStr">
@@ -20697,6 +21264,11 @@
       <c r="Q120" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R120" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="35.05" customHeight="1" s="32">
       <c r="A121" s="55" t="inlineStr">
@@ -20777,6 +21349,11 @@
       <c r="Q121" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R121" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="23.85" customHeight="1" s="32">
       <c r="A122" s="55" t="inlineStr">
@@ -20857,6 +21434,11 @@
       <c r="Q122" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R122" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="23.85" customHeight="1" s="32">
       <c r="A123" s="49" t="inlineStr">
@@ -20937,6 +21519,11 @@
       <c r="Q123" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R123" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="23.85" customHeight="1" s="32">
       <c r="A124" s="55" t="inlineStr">
@@ -21017,6 +21604,11 @@
       <c r="Q124" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R124" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="23.85" customHeight="1" s="32">
       <c r="A125" s="55" t="inlineStr">
@@ -21097,6 +21689,11 @@
       <c r="Q125" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R125" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="23.85" customHeight="1" s="32">
       <c r="A126" s="49" t="inlineStr">
@@ -21177,6 +21774,11 @@
       <c r="Q126" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R126" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="23.85" customHeight="1" s="32">
       <c r="A127" s="49" t="inlineStr">
@@ -21257,6 +21859,11 @@
       <c r="Q127" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R127" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="23.85" customHeight="1" s="32">
       <c r="A128" s="55" t="inlineStr">
@@ -21337,6 +21944,11 @@
       <c r="Q128" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R128" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="23.85" customHeight="1" s="32">
       <c r="A129" s="49" t="inlineStr">
@@ -21417,6 +22029,11 @@
       <c r="Q129" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R129" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="23.85" customHeight="1" s="32">
       <c r="A130" s="55" t="inlineStr">
@@ -21497,6 +22114,11 @@
       <c r="Q130" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R130" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="23.85" customHeight="1" s="32">
       <c r="A131" s="49" t="inlineStr">
@@ -21577,6 +22199,11 @@
       <c r="Q131" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R131" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="23.85" customHeight="1" s="32">
       <c r="A132" s="45" t="inlineStr">
@@ -21657,6 +22284,11 @@
       <c r="Q132" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R132" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="23.85" customHeight="1" s="32">
       <c r="A133" s="45" t="inlineStr">
@@ -21737,6 +22369,11 @@
       <c r="Q133" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R133" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="23.85" customHeight="1" s="32">
       <c r="A134" s="55" t="inlineStr">
@@ -21817,6 +22454,11 @@
       <c r="Q134" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R134" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="23.85" customHeight="1" s="32">
       <c r="A135" s="55" t="inlineStr">
@@ -21897,6 +22539,11 @@
       <c r="Q135" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R135" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="23.85" customHeight="1" s="32">
       <c r="A136" s="55" t="inlineStr">
@@ -21977,6 +22624,11 @@
       <c r="Q136" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R136" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="23.85" customHeight="1" s="32">
       <c r="A137" s="55" t="inlineStr">
@@ -22057,6 +22709,11 @@
       <c r="Q137" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R137" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="23.85" customHeight="1" s="32">
       <c r="A138" s="55" t="inlineStr">
@@ -22137,6 +22794,11 @@
       <c r="Q138" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R138" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="23.85" customHeight="1" s="32">
       <c r="A139" s="55" t="inlineStr">
@@ -22217,6 +22879,11 @@
       <c r="Q139" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R139" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="23.85" customHeight="1" s="32">
       <c r="A140" s="55" t="inlineStr">
@@ -22297,6 +22964,11 @@
       <c r="Q140" s="56" t="n">
         <v>10</v>
       </c>
+      <c r="R140" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="23.85" customHeight="1" s="32">
       <c r="A141" s="55" t="inlineStr">
@@ -22377,6 +23049,11 @@
       <c r="Q141" s="56" t="n">
         <v>5</v>
       </c>
+      <c r="R141" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="23.85" customHeight="1" s="32">
       <c r="A142" s="49" t="inlineStr">
@@ -22457,6 +23134,11 @@
       <c r="Q142" s="48" t="n">
         <v>60</v>
       </c>
+      <c r="R142" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="23.85" customHeight="1" s="32">
       <c r="A143" s="55" t="inlineStr">
@@ -22537,6 +23219,11 @@
       <c r="Q143" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R143" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="23.85" customHeight="1" s="32">
       <c r="A144" s="45" t="inlineStr">
@@ -22617,6 +23304,11 @@
       <c r="Q144" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R144" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="23.85" customHeight="1" s="32">
       <c r="A145" s="45" t="inlineStr">
@@ -22697,6 +23389,11 @@
       <c r="Q145" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R145" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="23.85" customHeight="1" s="32">
       <c r="A146" s="45" t="inlineStr">
@@ -22777,6 +23474,11 @@
       <c r="Q146" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R146" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="35.05" customHeight="1" s="32">
       <c r="A147" s="49" t="inlineStr">
@@ -22857,6 +23559,11 @@
       <c r="Q147" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R147" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="23.85" customHeight="1" s="32">
       <c r="A148" s="45" t="inlineStr">
@@ -22937,6 +23644,11 @@
       <c r="Q148" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R148" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="23.85" customHeight="1" s="32">
       <c r="A149" s="55" t="inlineStr">
@@ -23017,6 +23729,11 @@
       <c r="Q149" s="56" t="n">
         <v>20</v>
       </c>
+      <c r="R149" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="23.85" customHeight="1" s="32">
       <c r="A150" s="55" t="inlineStr">
@@ -23097,6 +23814,11 @@
       <c r="Q150" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R150" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="23.85" customHeight="1" s="32">
       <c r="A151" s="55" t="inlineStr">
@@ -23177,6 +23899,11 @@
       <c r="Q151" s="56" t="n">
         <v>45</v>
       </c>
+      <c r="R151" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="23.85" customHeight="1" s="32">
       <c r="A152" s="49" t="inlineStr">
@@ -23257,6 +23984,11 @@
       <c r="Q152" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R152" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="23.85" customHeight="1" s="32">
       <c r="A153" s="55" t="inlineStr">
@@ -23337,6 +24069,11 @@
       <c r="Q153" s="56" t="n">
         <v>15</v>
       </c>
+      <c r="R153" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="23.85" customHeight="1" s="32">
       <c r="A154" s="55" t="inlineStr">
@@ -23417,6 +24154,11 @@
       <c r="Q154" s="56" t="n">
         <v>45</v>
       </c>
+      <c r="R154" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="23.85" customHeight="1" s="32">
       <c r="A155" s="55" t="inlineStr">
@@ -23497,6 +24239,11 @@
       <c r="Q155" s="56" t="n">
         <v>180</v>
       </c>
+      <c r="R155" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="23.85" customHeight="1" s="32">
       <c r="A156" s="55" t="inlineStr">
@@ -23577,6 +24324,11 @@
       <c r="Q156" s="56" t="n">
         <v>30</v>
       </c>
+      <c r="R156" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="35.05" customHeight="1" s="32">
       <c r="A157" s="49" t="inlineStr">
@@ -23657,6 +24409,11 @@
       <c r="Q157" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R157" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="35.05" customHeight="1" s="32">
       <c r="A158" s="49" t="inlineStr">
@@ -23737,6 +24494,11 @@
       <c r="Q158" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R158" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="159" ht="35.05" customHeight="1" s="32">
       <c r="A159" s="45" t="inlineStr">
@@ -23817,6 +24579,11 @@
       <c r="Q159" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="R159" s="59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="49" t="inlineStr">
@@ -23897,6 +24664,11 @@
       <c r="Q160" s="48" t="n">
         <v>2</v>
       </c>
+      <c r="R160" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="49" t="inlineStr">
@@ -23977,6 +24749,11 @@
       <c r="Q161" s="48" t="n">
         <v>15</v>
       </c>
+      <c r="R161" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="49" t="inlineStr">
@@ -24057,6 +24834,11 @@
       <c r="Q162" s="48" t="n">
         <v>0</v>
       </c>
+      <c r="R162" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="49" t="inlineStr">
@@ -24116,7 +24898,7 @@
       </c>
       <c r="M163" s="51" t="inlineStr">
         <is>
-          <t>Un détecteur non conforme peut ne pas être reconnu par l'assureur</t>
+          <t>Un détecteur non conforme peut ne pas être reconnu par votre assureur</t>
         </is>
       </c>
       <c r="N163" s="49" t="inlineStr">
@@ -24136,6 +24918,11 @@
       </c>
       <c r="Q163" s="48" t="n">
         <v>5</v>
+      </c>
+      <c r="R163" s="48" t="inlineStr">
+        <is>
+          <t>Un détecteur non conforme peut ne pas être reconnu par votre assureur</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -24152,7 +24939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N90"/>
+  <dimension ref="A2:N90"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="31" min="1" max="1"/>
@@ -24168,7 +24955,6 @@
     <col width="30" customWidth="1" style="31" min="12" max="13"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="19.7" customHeight="1" s="32">
       <c r="A2" s="33" t="inlineStr">
         <is>
@@ -24183,7 +24969,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="32">
       <c r="A5" s="41" t="inlineStr">
         <is>
@@ -30220,7 +31005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A2:I45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="31" min="1" max="2"/>
@@ -30231,7 +31016,6 @@
     <col width="60" customWidth="1" style="31" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="19.7" customHeight="1" s="32">
       <c r="A2" s="33" t="inlineStr">
         <is>
@@ -30246,7 +31030,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="32">
       <c r="A5" s="41" t="inlineStr">
         <is>
@@ -30288,6 +31071,11 @@
           <t>Conseil si a confirmer</t>
         </is>
       </c>
+      <c r="I5" s="41" t="inlineStr">
+        <is>
+          <t>Conseil si en retard</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="32">
       <c r="A6" s="48" t="inlineStr">
@@ -30330,6 +31118,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I6" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="32">
       <c r="A7" s="48" t="inlineStr">
@@ -30372,6 +31165,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I7" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="32">
       <c r="A8" s="48" t="inlineStr">
@@ -30414,6 +31212,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I8" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="32">
       <c r="A9" s="48" t="inlineStr">
@@ -30456,6 +31259,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I9" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="32">
       <c r="A10" s="48" t="inlineStr">
@@ -30498,6 +31306,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I10" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="23.85" customHeight="1" s="32">
       <c r="A11" s="48" t="inlineStr">
@@ -30540,6 +31353,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I11" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="32">
       <c r="A12" s="48" t="inlineStr">
@@ -30582,6 +31400,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I12" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="23.85" customHeight="1" s="32">
       <c r="A13" s="48" t="inlineStr">
@@ -30624,6 +31447,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I13" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="23.85" customHeight="1" s="32">
       <c r="A14" s="48" t="inlineStr">
@@ -30666,6 +31494,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I14" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="23.85" customHeight="1" s="32">
       <c r="A15" s="48" t="inlineStr">
@@ -30708,6 +31541,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I15" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="23.85" customHeight="1" s="32">
       <c r="A16" s="48" t="inlineStr">
@@ -30750,6 +31588,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I16" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="23.85" customHeight="1" s="32">
       <c r="A17" s="48" t="inlineStr">
@@ -30792,6 +31635,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I17" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="23.85" customHeight="1" s="32">
       <c r="A18" s="48" t="inlineStr">
@@ -30834,6 +31682,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I18" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="23.85" customHeight="1" s="32">
       <c r="A19" s="48" t="inlineStr">
@@ -30876,6 +31729,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I19" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="23.85" customHeight="1" s="32">
       <c r="A20" s="48" t="inlineStr">
@@ -30918,6 +31776,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I20" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="23.85" customHeight="1" s="32">
       <c r="A21" s="48" t="inlineStr">
@@ -30960,6 +31823,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I21" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="23.85" customHeight="1" s="32">
       <c r="A22" s="48" t="inlineStr">
@@ -31002,6 +31870,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I22" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="32">
       <c r="A23" s="48" t="inlineStr">
@@ -31044,6 +31917,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I23" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="23.85" customHeight="1" s="32">
       <c r="A24" s="48" t="inlineStr">
@@ -31086,6 +31964,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I24" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="23.85" customHeight="1" s="32">
       <c r="A25" s="48" t="inlineStr">
@@ -31128,6 +32011,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I25" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="23.85" customHeight="1" s="32">
       <c r="A26" s="48" t="inlineStr">
@@ -31170,6 +32058,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I26" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="32">
       <c r="A27" s="48" t="inlineStr">
@@ -31212,6 +32105,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I27" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="23.85" customHeight="1" s="32">
       <c r="A28" s="48" t="inlineStr">
@@ -31254,6 +32152,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I28" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="32">
       <c r="A29" s="48" t="inlineStr">
@@ -31296,6 +32199,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I29" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="32">
       <c r="A30" s="48" t="inlineStr">
@@ -31338,6 +32246,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I30" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="32">
       <c r="A31" s="48" t="inlineStr">
@@ -31380,6 +32293,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I31" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="35.05" customHeight="1" s="32">
       <c r="A32" s="48" t="inlineStr">
@@ -31422,6 +32340,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I32" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="46.25" customHeight="1" s="32">
       <c r="A33" s="48" t="inlineStr">
@@ -31464,6 +32387,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I33" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="23.85" customHeight="1" s="32">
       <c r="A34" s="48" t="inlineStr">
@@ -31506,6 +32434,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I34" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="23.85" customHeight="1" s="32">
       <c r="A35" s="48" t="inlineStr">
@@ -31548,6 +32481,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I35" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="23.85" customHeight="1" s="32">
       <c r="A36" s="48" t="inlineStr">
@@ -31590,6 +32528,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I36" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="32">
       <c r="A37" s="61" t="inlineStr">
@@ -31632,6 +32575,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I37" s="53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="32">
       <c r="A38" s="61" t="inlineStr">
@@ -31674,6 +32622,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I38" s="53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="23.85" customHeight="1" s="32">
       <c r="A39" s="61" t="inlineStr">
@@ -31716,6 +32669,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I39" s="53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="32">
       <c r="A40" s="61" t="inlineStr">
@@ -31758,6 +32716,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I40" s="53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="23.85" customHeight="1" s="32">
       <c r="A41" s="61" t="inlineStr">
@@ -31800,6 +32763,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I41" s="53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="61" t="inlineStr">
@@ -31842,6 +32810,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I42" s="53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="48" t="inlineStr">
@@ -31884,6 +32857,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I43" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="61" t="inlineStr">
@@ -31926,6 +32904,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I44" s="53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="48" t="inlineStr">
@@ -31966,6 +32949,11 @@
       <c r="H45" s="51" t="inlineStr">
         <is>
           <t>Regardez l'étiquette au dos du détecteur, ou le contrat de télésurveillance.</t>
+        </is>
+      </c>
+      <c r="I45" s="51" t="inlineStr">
+        <is>
+          <t>Remplacez le détecteur par un modèle conforme, ou contactez votre prestataire de télésurveillance.</t>
         </is>
       </c>
     </row>
@@ -32961,7 +33949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A2:N26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="31" min="1" max="1"/>
@@ -32978,7 +33966,6 @@
     <col width="40" customWidth="1" style="31" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="19.7" customHeight="1" s="32">
       <c r="A2" s="33" t="inlineStr">
         <is>
@@ -32993,7 +33980,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="32">
       <c r="A5" s="41" t="inlineStr">
         <is>

</xml_diff>